<commit_message>
Fix birth date formatting to DD/MM/YYYY and impement nationality detection in Excel import modules
</commit_message>
<xml_diff>
--- a/BASE DATOS MODO APS.xlsx
+++ b/BASE DATOS MODO APS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanvidalp/Documents/clon carrera funcionaria/carrera-aps-digital/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B112CC2A-96BF-EE4A-90E2-8984ECD6D2CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A4FF23-A9AB-8F4C-8CC6-159B411B38CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30240" yWindow="1480" windowWidth="30240" windowHeight="18980" xr2:uid="{A9505C21-DF7A-114D-A7E6-2CB0B98403BE}"/>
   </bookViews>
@@ -2826,9 +2826,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
-  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -2880,17 +2877,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3233,7 +3229,7 @@
     <col min="3" max="3" width="39.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.5" customWidth="1"/>
-    <col min="8" max="8" width="19.83203125" style="6" customWidth="1"/>
+    <col min="8" max="8" width="19.1640625" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -3278,7 +3274,7 @@
       <c r="E2" s="1" t="s">
         <v>513</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="1" t="s">
         <v>532</v>
       </c>
       <c r="G2" s="1" t="s">

</xml_diff>

<commit_message>
Fix field mapping: sync birth_date, nationality and include position in validation
</commit_message>
<xml_diff>
--- a/BASE DATOS MODO APS.xlsx
+++ b/BASE DATOS MODO APS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juanvidalp/Documents/clon carrera funcionaria/carrera-aps-digital/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A4FF23-A9AB-8F4C-8CC6-159B411B38CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B103A0-598C-2349-9DA3-E57CE6A575F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30240" yWindow="1480" windowWidth="30240" windowHeight="18980" xr2:uid="{A9505C21-DF7A-114D-A7E6-2CB0B98403BE}"/>
   </bookViews>
@@ -2826,6 +2826,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -2877,21 +2880,154 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="8">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -2902,6 +3038,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{295653C2-543A-3242-AC88-B07A27B84D8D}" name="Tabla2" displayName="Tabla2" ref="A1:H442" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:H442" xr:uid="{295653C2-543A-3242-AC88-B07A27B84D8D}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{B37AE236-64D2-614F-995B-667452BE6B5F}" name="RUT" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{A61045C6-6455-9B46-B60D-6273BA4D7AEA}" name="NOMBRE"/>
+    <tableColumn id="3" xr3:uid="{AF558316-47E5-FE45-A078-9EF04A4DFC4B}" name="Establecimiento" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{F3DFD452-EA04-D749-B980-7F229697155D}" name="Categoría" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{D1D00D42-53FA-F44A-82B4-5776848CF6FD}" name=" Profesión" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{56286FD2-BD2C-B24F-BC6D-CA7C58A5C9B3}" name="Nacionalidad" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{A0198422-0804-DD43-9BD8-F5191267A456}" name="Tipo Contrato" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{E5EB52D8-7F4C-ED44-AA40-35686055C1FA}" name="Fecha Nacimiento" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3224,16 +3377,17 @@
   <dimension ref="A1:H442"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.1640625" customWidth="1"/>
+    <col min="1" max="1" width="22.1640625" style="8" customWidth="1"/>
     <col min="2" max="2" width="38.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="39.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="23" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.5" customWidth="1"/>
-    <col min="8" max="8" width="19.1640625" style="6" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -3259,7 +3413,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B2" t="s">
@@ -3285,7 +3439,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B3" t="s">
@@ -3311,7 +3465,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="8" t="s">
         <v>22</v>
       </c>
       <c r="B4" t="s">
@@ -3337,7 +3491,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="8" t="s">
         <v>23</v>
       </c>
       <c r="B5" t="s">
@@ -3363,7 +3517,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="8" t="s">
         <v>24</v>
       </c>
       <c r="B6" t="s">
@@ -3389,7 +3543,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="8" t="s">
         <v>25</v>
       </c>
       <c r="B7" t="s">
@@ -3415,7 +3569,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="8" t="s">
         <v>26</v>
       </c>
       <c r="B8" t="s">
@@ -3441,7 +3595,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="8" t="s">
         <v>27</v>
       </c>
       <c r="B9" t="s">
@@ -3467,7 +3621,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="A10" s="8" t="s">
         <v>28</v>
       </c>
       <c r="B10" t="s">
@@ -3493,7 +3647,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="8" t="s">
         <v>29</v>
       </c>
       <c r="B11" t="s">
@@ -3519,7 +3673,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="A12" s="8" t="s">
         <v>30</v>
       </c>
       <c r="B12" t="s">
@@ -3545,7 +3699,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="A13" s="8" t="s">
         <v>31</v>
       </c>
       <c r="B13" t="s">
@@ -3571,7 +3725,7 @@
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="A14" s="8" t="s">
         <v>32</v>
       </c>
       <c r="B14" t="s">
@@ -3597,7 +3751,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="A15" s="8" t="s">
         <v>33</v>
       </c>
       <c r="B15" t="s">
@@ -3623,7 +3777,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="A16" s="8" t="s">
         <v>34</v>
       </c>
       <c r="B16" t="s">
@@ -3649,7 +3803,7 @@
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="A17" s="8" t="s">
         <v>35</v>
       </c>
       <c r="B17" t="s">
@@ -3675,7 +3829,7 @@
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="A18" s="8" t="s">
         <v>36</v>
       </c>
       <c r="B18" t="s">
@@ -3701,7 +3855,7 @@
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="A19" s="8" t="s">
         <v>37</v>
       </c>
       <c r="B19" t="s">
@@ -3727,7 +3881,7 @@
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="A20" s="8" t="s">
         <v>38</v>
       </c>
       <c r="B20" t="s">
@@ -3753,7 +3907,7 @@
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="A21" s="8" t="s">
         <v>39</v>
       </c>
       <c r="B21" t="s">
@@ -3779,7 +3933,7 @@
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="A22" s="8" t="s">
         <v>40</v>
       </c>
       <c r="B22" t="s">
@@ -3805,7 +3959,7 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="A23" s="8" t="s">
         <v>41</v>
       </c>
       <c r="B23" t="s">
@@ -3831,7 +3985,7 @@
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="A24" s="8" t="s">
         <v>42</v>
       </c>
       <c r="B24" t="s">
@@ -3857,7 +4011,7 @@
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="A25" s="8" t="s">
         <v>43</v>
       </c>
       <c r="B25" t="s">
@@ -3883,7 +4037,7 @@
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="A26" s="8" t="s">
         <v>44</v>
       </c>
       <c r="B26" t="s">
@@ -3909,7 +4063,7 @@
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="A27" s="8" t="s">
         <v>45</v>
       </c>
       <c r="B27" t="s">
@@ -3935,7 +4089,7 @@
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="A28" s="8" t="s">
         <v>46</v>
       </c>
       <c r="B28" t="s">
@@ -3961,7 +4115,7 @@
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+      <c r="A29" s="8" t="s">
         <v>47</v>
       </c>
       <c r="B29" t="s">
@@ -3987,7 +4141,7 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+      <c r="A30" s="8" t="s">
         <v>48</v>
       </c>
       <c r="B30" t="s">
@@ -4013,7 +4167,7 @@
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+      <c r="A31" s="8" t="s">
         <v>49</v>
       </c>
       <c r="B31" t="s">
@@ -4039,7 +4193,7 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+      <c r="A32" s="8" t="s">
         <v>50</v>
       </c>
       <c r="B32" t="s">
@@ -4065,7 +4219,7 @@
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+      <c r="A33" s="8" t="s">
         <v>51</v>
       </c>
       <c r="B33" t="s">
@@ -4091,7 +4245,7 @@
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="A34" s="8" t="s">
         <v>52</v>
       </c>
       <c r="B34" t="s">
@@ -4117,7 +4271,7 @@
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="A35" s="8" t="s">
         <v>53</v>
       </c>
       <c r="B35" t="s">
@@ -4143,7 +4297,7 @@
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+      <c r="A36" s="8" t="s">
         <v>54</v>
       </c>
       <c r="B36" t="s">
@@ -4169,7 +4323,7 @@
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+      <c r="A37" s="8" t="s">
         <v>55</v>
       </c>
       <c r="B37" t="s">
@@ -4195,7 +4349,7 @@
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+      <c r="A38" s="8" t="s">
         <v>56</v>
       </c>
       <c r="B38" t="s">
@@ -4221,7 +4375,7 @@
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+      <c r="A39" s="8" t="s">
         <v>57</v>
       </c>
       <c r="B39" t="s">
@@ -4247,7 +4401,7 @@
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="A40" s="8" t="s">
         <v>58</v>
       </c>
       <c r="B40" t="s">
@@ -4273,7 +4427,7 @@
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="A41" s="8" t="s">
         <v>59</v>
       </c>
       <c r="B41" t="s">
@@ -4299,7 +4453,7 @@
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+      <c r="A42" s="8" t="s">
         <v>60</v>
       </c>
       <c r="B42" t="s">
@@ -4325,7 +4479,7 @@
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+      <c r="A43" s="8" t="s">
         <v>61</v>
       </c>
       <c r="B43" t="s">
@@ -4351,7 +4505,7 @@
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="A44" s="8" t="s">
         <v>62</v>
       </c>
       <c r="B44" t="s">
@@ -4377,7 +4531,7 @@
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+      <c r="A45" s="8" t="s">
         <v>63</v>
       </c>
       <c r="B45" t="s">
@@ -4403,7 +4557,7 @@
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="A46" s="8" t="s">
         <v>64</v>
       </c>
       <c r="B46" t="s">
@@ -4429,7 +4583,7 @@
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+      <c r="A47" s="8" t="s">
         <v>65</v>
       </c>
       <c r="B47" t="s">
@@ -4455,7 +4609,7 @@
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+      <c r="A48" s="8" t="s">
         <v>66</v>
       </c>
       <c r="B48" t="s">
@@ -4481,7 +4635,7 @@
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+      <c r="A49" s="8" t="s">
         <v>67</v>
       </c>
       <c r="B49" t="s">
@@ -4507,7 +4661,7 @@
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+      <c r="A50" s="8" t="s">
         <v>68</v>
       </c>
       <c r="B50" t="s">
@@ -4533,7 +4687,7 @@
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+      <c r="A51" s="8" t="s">
         <v>69</v>
       </c>
       <c r="B51" t="s">
@@ -4559,7 +4713,7 @@
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+      <c r="A52" s="8" t="s">
         <v>70</v>
       </c>
       <c r="B52" t="s">
@@ -4585,7 +4739,7 @@
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+      <c r="A53" s="8" t="s">
         <v>71</v>
       </c>
       <c r="B53" t="s">
@@ -4611,7 +4765,7 @@
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+      <c r="A54" s="8" t="s">
         <v>72</v>
       </c>
       <c r="B54" t="s">
@@ -4637,7 +4791,7 @@
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
+      <c r="A55" s="8" t="s">
         <v>73</v>
       </c>
       <c r="B55" t="s">
@@ -4663,7 +4817,7 @@
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+      <c r="A56" s="8" t="s">
         <v>74</v>
       </c>
       <c r="B56" t="s">
@@ -4689,7 +4843,7 @@
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+      <c r="A57" s="8" t="s">
         <v>75</v>
       </c>
       <c r="B57" t="s">
@@ -4715,7 +4869,7 @@
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
+      <c r="A58" s="8" t="s">
         <v>76</v>
       </c>
       <c r="B58" t="s">
@@ -4741,7 +4895,7 @@
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
+      <c r="A59" s="8" t="s">
         <v>77</v>
       </c>
       <c r="B59" t="s">
@@ -4767,7 +4921,7 @@
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
+      <c r="A60" s="8" t="s">
         <v>78</v>
       </c>
       <c r="B60" t="s">
@@ -4793,7 +4947,7 @@
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
+      <c r="A61" s="8" t="s">
         <v>79</v>
       </c>
       <c r="B61" t="s">
@@ -4819,7 +4973,7 @@
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
+      <c r="A62" s="8" t="s">
         <v>79</v>
       </c>
       <c r="B62" t="s">
@@ -4845,7 +4999,7 @@
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
+      <c r="A63" s="8" t="s">
         <v>80</v>
       </c>
       <c r="B63" t="s">
@@ -4871,7 +5025,7 @@
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
+      <c r="A64" s="8" t="s">
         <v>81</v>
       </c>
       <c r="B64" t="s">
@@ -4897,7 +5051,7 @@
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
+      <c r="A65" s="8" t="s">
         <v>82</v>
       </c>
       <c r="B65" t="s">
@@ -4923,7 +5077,7 @@
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
+      <c r="A66" s="8" t="s">
         <v>83</v>
       </c>
       <c r="B66" t="s">
@@ -4949,7 +5103,7 @@
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
+      <c r="A67" s="8" t="s">
         <v>84</v>
       </c>
       <c r="B67" t="s">
@@ -4975,7 +5129,7 @@
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
+      <c r="A68" s="8" t="s">
         <v>85</v>
       </c>
       <c r="B68" t="s">
@@ -5001,7 +5155,7 @@
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
+      <c r="A69" s="8" t="s">
         <v>86</v>
       </c>
       <c r="B69" t="s">
@@ -5027,7 +5181,7 @@
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
+      <c r="A70" s="8" t="s">
         <v>87</v>
       </c>
       <c r="B70" t="s">
@@ -5053,7 +5207,7 @@
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
+      <c r="A71" s="8" t="s">
         <v>88</v>
       </c>
       <c r="B71" t="s">
@@ -5079,7 +5233,7 @@
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
+      <c r="A72" s="8" t="s">
         <v>89</v>
       </c>
       <c r="B72" t="s">
@@ -5105,7 +5259,7 @@
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
+      <c r="A73" s="8" t="s">
         <v>90</v>
       </c>
       <c r="B73" t="s">
@@ -5131,7 +5285,7 @@
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
+      <c r="A74" s="8" t="s">
         <v>91</v>
       </c>
       <c r="B74" t="s">
@@ -5157,7 +5311,7 @@
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
+      <c r="A75" s="8" t="s">
         <v>92</v>
       </c>
       <c r="B75" t="s">
@@ -5183,7 +5337,7 @@
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
+      <c r="A76" s="8" t="s">
         <v>93</v>
       </c>
       <c r="B76" t="s">
@@ -5209,7 +5363,7 @@
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
+      <c r="A77" s="8" t="s">
         <v>94</v>
       </c>
       <c r="B77" t="s">
@@ -5235,7 +5389,7 @@
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A78" t="s">
+      <c r="A78" s="8" t="s">
         <v>95</v>
       </c>
       <c r="B78" t="s">
@@ -5261,7 +5415,7 @@
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A79" t="s">
+      <c r="A79" s="8" t="s">
         <v>96</v>
       </c>
       <c r="B79" t="s">
@@ -5287,7 +5441,7 @@
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
+      <c r="A80" s="8" t="s">
         <v>97</v>
       </c>
       <c r="B80" t="s">
@@ -5313,7 +5467,7 @@
       </c>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
+      <c r="A81" s="8" t="s">
         <v>98</v>
       </c>
       <c r="B81" t="s">
@@ -5339,7 +5493,7 @@
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
+      <c r="A82" s="8" t="s">
         <v>99</v>
       </c>
       <c r="B82" t="s">
@@ -5365,7 +5519,7 @@
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A83" t="s">
+      <c r="A83" s="8" t="s">
         <v>100</v>
       </c>
       <c r="B83" t="s">
@@ -5391,7 +5545,7 @@
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
+      <c r="A84" s="8" t="s">
         <v>101</v>
       </c>
       <c r="B84" t="s">
@@ -5417,7 +5571,7 @@
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
+      <c r="A85" s="8" t="s">
         <v>102</v>
       </c>
       <c r="B85" t="s">
@@ -5443,7 +5597,7 @@
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
+      <c r="A86" s="8" t="s">
         <v>103</v>
       </c>
       <c r="B86" t="s">
@@ -5469,7 +5623,7 @@
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
+      <c r="A87" s="8" t="s">
         <v>104</v>
       </c>
       <c r="B87" t="s">
@@ -5495,7 +5649,7 @@
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
+      <c r="A88" s="8" t="s">
         <v>105</v>
       </c>
       <c r="B88" t="s">
@@ -5521,7 +5675,7 @@
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A89" t="s">
+      <c r="A89" s="8" t="s">
         <v>106</v>
       </c>
       <c r="B89" t="s">
@@ -5547,7 +5701,7 @@
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
+      <c r="A90" s="8" t="s">
         <v>107</v>
       </c>
       <c r="B90" t="s">
@@ -5573,7 +5727,7 @@
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
+      <c r="A91" s="8" t="s">
         <v>108</v>
       </c>
       <c r="B91" t="s">
@@ -5599,7 +5753,7 @@
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
+      <c r="A92" s="8" t="s">
         <v>109</v>
       </c>
       <c r="B92" t="s">
@@ -5625,7 +5779,7 @@
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
+      <c r="A93" s="8" t="s">
         <v>110</v>
       </c>
       <c r="B93" t="s">
@@ -5651,7 +5805,7 @@
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
+      <c r="A94" s="8" t="s">
         <v>111</v>
       </c>
       <c r="B94" t="s">
@@ -5677,7 +5831,7 @@
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
+      <c r="A95" s="8" t="s">
         <v>112</v>
       </c>
       <c r="B95" t="s">
@@ -5703,7 +5857,7 @@
       </c>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A96" t="s">
+      <c r="A96" s="8" t="s">
         <v>113</v>
       </c>
       <c r="B96" t="s">
@@ -5729,7 +5883,7 @@
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A97" t="s">
+      <c r="A97" s="8" t="s">
         <v>114</v>
       </c>
       <c r="B97" t="s">
@@ -5755,7 +5909,7 @@
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
+      <c r="A98" s="8" t="s">
         <v>115</v>
       </c>
       <c r="B98" t="s">
@@ -5781,7 +5935,7 @@
       </c>
     </row>
     <row r="99" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A99" t="s">
+      <c r="A99" s="8" t="s">
         <v>116</v>
       </c>
       <c r="B99" t="s">
@@ -5807,7 +5961,7 @@
       </c>
     </row>
     <row r="100" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A100" t="s">
+      <c r="A100" s="8" t="s">
         <v>117</v>
       </c>
       <c r="B100" t="s">
@@ -5833,7 +5987,7 @@
       </c>
     </row>
     <row r="101" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A101" t="s">
+      <c r="A101" s="8" t="s">
         <v>118</v>
       </c>
       <c r="B101" t="s">
@@ -5859,7 +6013,7 @@
       </c>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A102" t="s">
+      <c r="A102" s="8" t="s">
         <v>119</v>
       </c>
       <c r="B102" t="s">
@@ -5885,7 +6039,7 @@
       </c>
     </row>
     <row r="103" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
+      <c r="A103" s="8" t="s">
         <v>120</v>
       </c>
       <c r="B103" t="s">
@@ -5911,7 +6065,7 @@
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
+      <c r="A104" s="8" t="s">
         <v>121</v>
       </c>
       <c r="B104" t="s">
@@ -5937,7 +6091,7 @@
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
+      <c r="A105" s="8" t="s">
         <v>122</v>
       </c>
       <c r="B105" t="s">
@@ -5963,7 +6117,7 @@
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
+      <c r="A106" s="8" t="s">
         <v>123</v>
       </c>
       <c r="B106" t="s">
@@ -5989,7 +6143,7 @@
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A107" t="s">
+      <c r="A107" s="8" t="s">
         <v>124</v>
       </c>
       <c r="B107" t="s">
@@ -6015,7 +6169,7 @@
       </c>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A108" t="s">
+      <c r="A108" s="8" t="s">
         <v>125</v>
       </c>
       <c r="B108" t="s">
@@ -6041,7 +6195,7 @@
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
+      <c r="A109" s="8" t="s">
         <v>126</v>
       </c>
       <c r="B109" t="s">
@@ -6067,7 +6221,7 @@
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A110" t="s">
+      <c r="A110" s="8" t="s">
         <v>127</v>
       </c>
       <c r="B110" t="s">
@@ -6093,7 +6247,7 @@
       </c>
     </row>
     <row r="111" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A111" t="s">
+      <c r="A111" s="8" t="s">
         <v>128</v>
       </c>
       <c r="B111" t="s">
@@ -6119,7 +6273,7 @@
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A112" t="s">
+      <c r="A112" s="8" t="s">
         <v>129</v>
       </c>
       <c r="B112" t="s">
@@ -6145,7 +6299,7 @@
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A113" t="s">
+      <c r="A113" s="8" t="s">
         <v>130</v>
       </c>
       <c r="B113" t="s">
@@ -6171,7 +6325,7 @@
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A114" t="s">
+      <c r="A114" s="8" t="s">
         <v>131</v>
       </c>
       <c r="B114" t="s">
@@ -6197,7 +6351,7 @@
       </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A115" t="s">
+      <c r="A115" s="8" t="s">
         <v>132</v>
       </c>
       <c r="B115" t="s">
@@ -6223,7 +6377,7 @@
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A116" t="s">
+      <c r="A116" s="8" t="s">
         <v>133</v>
       </c>
       <c r="B116" t="s">
@@ -6249,7 +6403,7 @@
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A117" t="s">
+      <c r="A117" s="8" t="s">
         <v>134</v>
       </c>
       <c r="B117" t="s">
@@ -6275,7 +6429,7 @@
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A118" t="s">
+      <c r="A118" s="8" t="s">
         <v>135</v>
       </c>
       <c r="B118" t="s">
@@ -6301,7 +6455,7 @@
       </c>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A119" t="s">
+      <c r="A119" s="8" t="s">
         <v>136</v>
       </c>
       <c r="B119" t="s">
@@ -6327,7 +6481,7 @@
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A120" t="s">
+      <c r="A120" s="8" t="s">
         <v>137</v>
       </c>
       <c r="B120" t="s">
@@ -6353,7 +6507,7 @@
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A121" t="s">
+      <c r="A121" s="8" t="s">
         <v>138</v>
       </c>
       <c r="B121" t="s">
@@ -6379,7 +6533,7 @@
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A122" t="s">
+      <c r="A122" s="8" t="s">
         <v>139</v>
       </c>
       <c r="B122" t="s">
@@ -6405,7 +6559,7 @@
       </c>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A123" t="s">
+      <c r="A123" s="8" t="s">
         <v>140</v>
       </c>
       <c r="B123" t="s">
@@ -6431,7 +6585,7 @@
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A124" t="s">
+      <c r="A124" s="8" t="s">
         <v>141</v>
       </c>
       <c r="B124" t="s">
@@ -6457,7 +6611,7 @@
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A125" t="s">
+      <c r="A125" s="8" t="s">
         <v>142</v>
       </c>
       <c r="B125" t="s">
@@ -6483,7 +6637,7 @@
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A126" t="s">
+      <c r="A126" s="8" t="s">
         <v>143</v>
       </c>
       <c r="B126" t="s">
@@ -6509,7 +6663,7 @@
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A127" t="s">
+      <c r="A127" s="8" t="s">
         <v>144</v>
       </c>
       <c r="B127" t="s">
@@ -6535,7 +6689,7 @@
       </c>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A128" t="s">
+      <c r="A128" s="8" t="s">
         <v>145</v>
       </c>
       <c r="B128" t="s">
@@ -6561,7 +6715,7 @@
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A129" t="s">
+      <c r="A129" s="8" t="s">
         <v>145</v>
       </c>
       <c r="B129" t="s">
@@ -6587,7 +6741,7 @@
       </c>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A130" t="s">
+      <c r="A130" s="8" t="s">
         <v>146</v>
       </c>
       <c r="B130" t="s">
@@ -6613,7 +6767,7 @@
       </c>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A131" t="s">
+      <c r="A131" s="8" t="s">
         <v>147</v>
       </c>
       <c r="B131" t="s">
@@ -6639,7 +6793,7 @@
       </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A132" t="s">
+      <c r="A132" s="8" t="s">
         <v>148</v>
       </c>
       <c r="B132" t="s">
@@ -6665,7 +6819,7 @@
       </c>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A133" t="s">
+      <c r="A133" s="8" t="s">
         <v>149</v>
       </c>
       <c r="B133" t="s">
@@ -6691,7 +6845,7 @@
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A134" t="s">
+      <c r="A134" s="8" t="s">
         <v>150</v>
       </c>
       <c r="B134" t="s">
@@ -6717,7 +6871,7 @@
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A135" t="s">
+      <c r="A135" s="8" t="s">
         <v>151</v>
       </c>
       <c r="B135" t="s">
@@ -6743,7 +6897,7 @@
       </c>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A136" t="s">
+      <c r="A136" s="8" t="s">
         <v>152</v>
       </c>
       <c r="B136" t="s">
@@ -6769,7 +6923,7 @@
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A137" t="s">
+      <c r="A137" s="8" t="s">
         <v>153</v>
       </c>
       <c r="B137" t="s">
@@ -6795,7 +6949,7 @@
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A138" t="s">
+      <c r="A138" s="8" t="s">
         <v>154</v>
       </c>
       <c r="B138" t="s">
@@ -6821,7 +6975,7 @@
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A139" t="s">
+      <c r="A139" s="8" t="s">
         <v>155</v>
       </c>
       <c r="B139" t="s">
@@ -6847,7 +7001,7 @@
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A140" t="s">
+      <c r="A140" s="8" t="s">
         <v>156</v>
       </c>
       <c r="B140" t="s">
@@ -6873,7 +7027,7 @@
       </c>
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A141" t="s">
+      <c r="A141" s="8" t="s">
         <v>157</v>
       </c>
       <c r="B141" t="s">
@@ -6899,7 +7053,7 @@
       </c>
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A142" t="s">
+      <c r="A142" s="8" t="s">
         <v>158</v>
       </c>
       <c r="B142" t="s">
@@ -6925,7 +7079,7 @@
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A143" t="s">
+      <c r="A143" s="8" t="s">
         <v>159</v>
       </c>
       <c r="B143" t="s">
@@ -6951,7 +7105,7 @@
       </c>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A144" t="s">
+      <c r="A144" s="8" t="s">
         <v>160</v>
       </c>
       <c r="B144" t="s">
@@ -6977,7 +7131,7 @@
       </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A145" t="s">
+      <c r="A145" s="8" t="s">
         <v>161</v>
       </c>
       <c r="B145" t="s">
@@ -7003,7 +7157,7 @@
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A146" t="s">
+      <c r="A146" s="8" t="s">
         <v>162</v>
       </c>
       <c r="B146" t="s">
@@ -7029,7 +7183,7 @@
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A147" t="s">
+      <c r="A147" s="8" t="s">
         <v>163</v>
       </c>
       <c r="B147" t="s">
@@ -7055,7 +7209,7 @@
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A148" t="s">
+      <c r="A148" s="8" t="s">
         <v>164</v>
       </c>
       <c r="B148" t="s">
@@ -7081,7 +7235,7 @@
       </c>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A149" t="s">
+      <c r="A149" s="8" t="s">
         <v>165</v>
       </c>
       <c r="B149" t="s">
@@ -7107,7 +7261,7 @@
       </c>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A150" t="s">
+      <c r="A150" s="8" t="s">
         <v>166</v>
       </c>
       <c r="B150" t="s">
@@ -7133,7 +7287,7 @@
       </c>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A151" t="s">
+      <c r="A151" s="8" t="s">
         <v>167</v>
       </c>
       <c r="B151" t="s">
@@ -7159,7 +7313,7 @@
       </c>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A152" t="s">
+      <c r="A152" s="8" t="s">
         <v>168</v>
       </c>
       <c r="B152" t="s">
@@ -7185,7 +7339,7 @@
       </c>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A153" t="s">
+      <c r="A153" s="8" t="s">
         <v>169</v>
       </c>
       <c r="B153" t="s">
@@ -7211,7 +7365,7 @@
       </c>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A154" t="s">
+      <c r="A154" s="8" t="s">
         <v>170</v>
       </c>
       <c r="B154" t="s">
@@ -7237,7 +7391,7 @@
       </c>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A155" t="s">
+      <c r="A155" s="8" t="s">
         <v>171</v>
       </c>
       <c r="B155" t="s">
@@ -7263,7 +7417,7 @@
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A156" t="s">
+      <c r="A156" s="8" t="s">
         <v>172</v>
       </c>
       <c r="B156" t="s">
@@ -7289,7 +7443,7 @@
       </c>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A157" t="s">
+      <c r="A157" s="8" t="s">
         <v>173</v>
       </c>
       <c r="B157" t="s">
@@ -7315,7 +7469,7 @@
       </c>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A158" t="s">
+      <c r="A158" s="8" t="s">
         <v>174</v>
       </c>
       <c r="B158" t="s">
@@ -7341,7 +7495,7 @@
       </c>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A159" t="s">
+      <c r="A159" s="8" t="s">
         <v>175</v>
       </c>
       <c r="B159" t="s">
@@ -7367,7 +7521,7 @@
       </c>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A160" t="s">
+      <c r="A160" s="8" t="s">
         <v>176</v>
       </c>
       <c r="B160" t="s">
@@ -7393,7 +7547,7 @@
       </c>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A161" t="s">
+      <c r="A161" s="8" t="s">
         <v>177</v>
       </c>
       <c r="B161" t="s">
@@ -7419,7 +7573,7 @@
       </c>
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A162" t="s">
+      <c r="A162" s="8" t="s">
         <v>178</v>
       </c>
       <c r="B162" t="s">
@@ -7445,7 +7599,7 @@
       </c>
     </row>
     <row r="163" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A163" t="s">
+      <c r="A163" s="8" t="s">
         <v>179</v>
       </c>
       <c r="B163" t="s">
@@ -7471,7 +7625,7 @@
       </c>
     </row>
     <row r="164" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A164" t="s">
+      <c r="A164" s="8" t="s">
         <v>180</v>
       </c>
       <c r="B164" t="s">
@@ -7497,7 +7651,7 @@
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A165" t="s">
+      <c r="A165" s="8" t="s">
         <v>181</v>
       </c>
       <c r="B165" t="s">
@@ -7523,7 +7677,7 @@
       </c>
     </row>
     <row r="166" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A166" t="s">
+      <c r="A166" s="8" t="s">
         <v>182</v>
       </c>
       <c r="B166" t="s">
@@ -7549,7 +7703,7 @@
       </c>
     </row>
     <row r="167" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A167" t="s">
+      <c r="A167" s="8" t="s">
         <v>183</v>
       </c>
       <c r="B167" t="s">
@@ -7575,7 +7729,7 @@
       </c>
     </row>
     <row r="168" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A168" t="s">
+      <c r="A168" s="8" t="s">
         <v>184</v>
       </c>
       <c r="B168" t="s">
@@ -7601,7 +7755,7 @@
       </c>
     </row>
     <row r="169" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A169" t="s">
+      <c r="A169" s="8" t="s">
         <v>185</v>
       </c>
       <c r="B169" t="s">
@@ -7627,7 +7781,7 @@
       </c>
     </row>
     <row r="170" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A170" t="s">
+      <c r="A170" s="8" t="s">
         <v>186</v>
       </c>
       <c r="B170" t="s">
@@ -7653,7 +7807,7 @@
       </c>
     </row>
     <row r="171" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A171" t="s">
+      <c r="A171" s="8" t="s">
         <v>187</v>
       </c>
       <c r="B171" t="s">
@@ -7679,7 +7833,7 @@
       </c>
     </row>
     <row r="172" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A172" t="s">
+      <c r="A172" s="8" t="s">
         <v>188</v>
       </c>
       <c r="B172" t="s">
@@ -7705,7 +7859,7 @@
       </c>
     </row>
     <row r="173" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A173" t="s">
+      <c r="A173" s="8" t="s">
         <v>189</v>
       </c>
       <c r="B173" t="s">
@@ -7731,7 +7885,7 @@
       </c>
     </row>
     <row r="174" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A174" t="s">
+      <c r="A174" s="8" t="s">
         <v>190</v>
       </c>
       <c r="B174" t="s">
@@ -7757,7 +7911,7 @@
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A175" t="s">
+      <c r="A175" s="8" t="s">
         <v>191</v>
       </c>
       <c r="B175" t="s">
@@ -7783,7 +7937,7 @@
       </c>
     </row>
     <row r="176" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A176" t="s">
+      <c r="A176" s="8" t="s">
         <v>192</v>
       </c>
       <c r="B176" t="s">
@@ -7809,7 +7963,7 @@
       </c>
     </row>
     <row r="177" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A177" t="s">
+      <c r="A177" s="8" t="s">
         <v>193</v>
       </c>
       <c r="B177" t="s">
@@ -7835,7 +7989,7 @@
       </c>
     </row>
     <row r="178" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A178" t="s">
+      <c r="A178" s="8" t="s">
         <v>194</v>
       </c>
       <c r="B178" t="s">
@@ -7861,7 +8015,7 @@
       </c>
     </row>
     <row r="179" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A179" t="s">
+      <c r="A179" s="8" t="s">
         <v>195</v>
       </c>
       <c r="B179" t="s">
@@ -7887,7 +8041,7 @@
       </c>
     </row>
     <row r="180" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A180" t="s">
+      <c r="A180" s="8" t="s">
         <v>196</v>
       </c>
       <c r="B180" t="s">
@@ -7913,7 +8067,7 @@
       </c>
     </row>
     <row r="181" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A181" t="s">
+      <c r="A181" s="8" t="s">
         <v>197</v>
       </c>
       <c r="B181" t="s">
@@ -7939,7 +8093,7 @@
       </c>
     </row>
     <row r="182" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A182" t="s">
+      <c r="A182" s="8" t="s">
         <v>198</v>
       </c>
       <c r="B182" t="s">
@@ -7965,7 +8119,7 @@
       </c>
     </row>
     <row r="183" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A183" t="s">
+      <c r="A183" s="8" t="s">
         <v>199</v>
       </c>
       <c r="B183" t="s">
@@ -7991,7 +8145,7 @@
       </c>
     </row>
     <row r="184" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A184" t="s">
+      <c r="A184" s="8" t="s">
         <v>200</v>
       </c>
       <c r="B184" t="s">
@@ -8017,7 +8171,7 @@
       </c>
     </row>
     <row r="185" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A185" t="s">
+      <c r="A185" s="8" t="s">
         <v>201</v>
       </c>
       <c r="B185" t="s">
@@ -8043,7 +8197,7 @@
       </c>
     </row>
     <row r="186" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A186" t="s">
+      <c r="A186" s="8" t="s">
         <v>202</v>
       </c>
       <c r="B186" t="s">
@@ -8069,7 +8223,7 @@
       </c>
     </row>
     <row r="187" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A187" t="s">
+      <c r="A187" s="8" t="s">
         <v>203</v>
       </c>
       <c r="B187" t="s">
@@ -8095,7 +8249,7 @@
       </c>
     </row>
     <row r="188" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A188" t="s">
+      <c r="A188" s="8" t="s">
         <v>204</v>
       </c>
       <c r="B188" t="s">
@@ -8121,7 +8275,7 @@
       </c>
     </row>
     <row r="189" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A189" t="s">
+      <c r="A189" s="8" t="s">
         <v>205</v>
       </c>
       <c r="B189" t="s">
@@ -8147,7 +8301,7 @@
       </c>
     </row>
     <row r="190" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A190" t="s">
+      <c r="A190" s="8" t="s">
         <v>206</v>
       </c>
       <c r="B190" t="s">
@@ -8173,7 +8327,7 @@
       </c>
     </row>
     <row r="191" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A191" t="s">
+      <c r="A191" s="8" t="s">
         <v>207</v>
       </c>
       <c r="B191" t="s">
@@ -8199,7 +8353,7 @@
       </c>
     </row>
     <row r="192" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A192" t="s">
+      <c r="A192" s="8" t="s">
         <v>208</v>
       </c>
       <c r="B192" t="s">
@@ -8225,7 +8379,7 @@
       </c>
     </row>
     <row r="193" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A193" t="s">
+      <c r="A193" s="8" t="s">
         <v>209</v>
       </c>
       <c r="B193" t="s">
@@ -8251,7 +8405,7 @@
       </c>
     </row>
     <row r="194" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A194" t="s">
+      <c r="A194" s="8" t="s">
         <v>210</v>
       </c>
       <c r="B194" t="s">
@@ -8277,7 +8431,7 @@
       </c>
     </row>
     <row r="195" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A195" t="s">
+      <c r="A195" s="8" t="s">
         <v>211</v>
       </c>
       <c r="B195" t="s">
@@ -8303,7 +8457,7 @@
       </c>
     </row>
     <row r="196" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A196" t="s">
+      <c r="A196" s="8" t="s">
         <v>212</v>
       </c>
       <c r="B196" t="s">
@@ -8329,7 +8483,7 @@
       </c>
     </row>
     <row r="197" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A197" t="s">
+      <c r="A197" s="8" t="s">
         <v>213</v>
       </c>
       <c r="B197" t="s">
@@ -8355,7 +8509,7 @@
       </c>
     </row>
     <row r="198" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A198" t="s">
+      <c r="A198" s="8" t="s">
         <v>214</v>
       </c>
       <c r="B198" t="s">
@@ -8381,7 +8535,7 @@
       </c>
     </row>
     <row r="199" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A199" t="s">
+      <c r="A199" s="8" t="s">
         <v>215</v>
       </c>
       <c r="B199" t="s">
@@ -8407,7 +8561,7 @@
       </c>
     </row>
     <row r="200" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A200" t="s">
+      <c r="A200" s="8" t="s">
         <v>216</v>
       </c>
       <c r="B200" t="s">
@@ -8433,7 +8587,7 @@
       </c>
     </row>
     <row r="201" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A201" t="s">
+      <c r="A201" s="8" t="s">
         <v>217</v>
       </c>
       <c r="B201" t="s">
@@ -8459,7 +8613,7 @@
       </c>
     </row>
     <row r="202" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A202" t="s">
+      <c r="A202" s="8" t="s">
         <v>218</v>
       </c>
       <c r="B202" t="s">
@@ -8485,7 +8639,7 @@
       </c>
     </row>
     <row r="203" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A203" t="s">
+      <c r="A203" s="8" t="s">
         <v>219</v>
       </c>
       <c r="B203" t="s">
@@ -8511,7 +8665,7 @@
       </c>
     </row>
     <row r="204" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A204" t="s">
+      <c r="A204" s="8" t="s">
         <v>220</v>
       </c>
       <c r="B204" t="s">
@@ -8537,7 +8691,7 @@
       </c>
     </row>
     <row r="205" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A205" t="s">
+      <c r="A205" s="8" t="s">
         <v>221</v>
       </c>
       <c r="B205" t="s">
@@ -8563,7 +8717,7 @@
       </c>
     </row>
     <row r="206" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A206" t="s">
+      <c r="A206" s="8" t="s">
         <v>222</v>
       </c>
       <c r="B206" t="s">
@@ -8589,7 +8743,7 @@
       </c>
     </row>
     <row r="207" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A207" t="s">
+      <c r="A207" s="8" t="s">
         <v>223</v>
       </c>
       <c r="B207" t="s">
@@ -8615,7 +8769,7 @@
       </c>
     </row>
     <row r="208" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A208" t="s">
+      <c r="A208" s="8" t="s">
         <v>224</v>
       </c>
       <c r="B208" t="s">
@@ -8641,7 +8795,7 @@
       </c>
     </row>
     <row r="209" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A209" t="s">
+      <c r="A209" s="8" t="s">
         <v>225</v>
       </c>
       <c r="B209" t="s">
@@ -8667,7 +8821,7 @@
       </c>
     </row>
     <row r="210" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A210" t="s">
+      <c r="A210" s="8" t="s">
         <v>226</v>
       </c>
       <c r="B210" t="s">
@@ -8693,7 +8847,7 @@
       </c>
     </row>
     <row r="211" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A211" t="s">
+      <c r="A211" s="8" t="s">
         <v>227</v>
       </c>
       <c r="B211" t="s">
@@ -8719,7 +8873,7 @@
       </c>
     </row>
     <row r="212" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A212" t="s">
+      <c r="A212" s="8" t="s">
         <v>228</v>
       </c>
       <c r="B212" t="s">
@@ -8745,7 +8899,7 @@
       </c>
     </row>
     <row r="213" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A213" t="s">
+      <c r="A213" s="8" t="s">
         <v>229</v>
       </c>
       <c r="B213" t="s">
@@ -8771,7 +8925,7 @@
       </c>
     </row>
     <row r="214" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A214" t="s">
+      <c r="A214" s="8" t="s">
         <v>230</v>
       </c>
       <c r="B214" t="s">
@@ -8797,7 +8951,7 @@
       </c>
     </row>
     <row r="215" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A215" t="s">
+      <c r="A215" s="8" t="s">
         <v>231</v>
       </c>
       <c r="B215" t="s">
@@ -8823,7 +8977,7 @@
       </c>
     </row>
     <row r="216" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A216" t="s">
+      <c r="A216" s="8" t="s">
         <v>232</v>
       </c>
       <c r="B216" t="s">
@@ -8849,7 +9003,7 @@
       </c>
     </row>
     <row r="217" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A217" t="s">
+      <c r="A217" s="8" t="s">
         <v>233</v>
       </c>
       <c r="B217" t="s">
@@ -8875,7 +9029,7 @@
       </c>
     </row>
     <row r="218" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A218" t="s">
+      <c r="A218" s="8" t="s">
         <v>234</v>
       </c>
       <c r="B218" t="s">
@@ -8901,7 +9055,7 @@
       </c>
     </row>
     <row r="219" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A219" t="s">
+      <c r="A219" s="8" t="s">
         <v>235</v>
       </c>
       <c r="B219" t="s">
@@ -8927,7 +9081,7 @@
       </c>
     </row>
     <row r="220" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A220" t="s">
+      <c r="A220" s="8" t="s">
         <v>236</v>
       </c>
       <c r="B220" t="s">
@@ -8953,7 +9107,7 @@
       </c>
     </row>
     <row r="221" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A221" t="s">
+      <c r="A221" s="8" t="s">
         <v>237</v>
       </c>
       <c r="B221" t="s">
@@ -8979,7 +9133,7 @@
       </c>
     </row>
     <row r="222" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A222" t="s">
+      <c r="A222" s="8" t="s">
         <v>238</v>
       </c>
       <c r="B222" t="s">
@@ -9005,7 +9159,7 @@
       </c>
     </row>
     <row r="223" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A223" t="s">
+      <c r="A223" s="8" t="s">
         <v>239</v>
       </c>
       <c r="B223" t="s">
@@ -9031,7 +9185,7 @@
       </c>
     </row>
     <row r="224" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A224" t="s">
+      <c r="A224" s="8" t="s">
         <v>240</v>
       </c>
       <c r="B224" t="s">
@@ -9057,7 +9211,7 @@
       </c>
     </row>
     <row r="225" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A225" t="s">
+      <c r="A225" s="8" t="s">
         <v>241</v>
       </c>
       <c r="B225" t="s">
@@ -9083,7 +9237,7 @@
       </c>
     </row>
     <row r="226" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A226" t="s">
+      <c r="A226" s="8" t="s">
         <v>242</v>
       </c>
       <c r="B226" t="s">
@@ -9109,7 +9263,7 @@
       </c>
     </row>
     <row r="227" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A227" t="s">
+      <c r="A227" s="8" t="s">
         <v>243</v>
       </c>
       <c r="B227" t="s">
@@ -9135,7 +9289,7 @@
       </c>
     </row>
     <row r="228" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A228" t="s">
+      <c r="A228" s="8" t="s">
         <v>244</v>
       </c>
       <c r="B228" t="s">
@@ -9161,7 +9315,7 @@
       </c>
     </row>
     <row r="229" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A229" t="s">
+      <c r="A229" s="8" t="s">
         <v>245</v>
       </c>
       <c r="B229" t="s">
@@ -9187,7 +9341,7 @@
       </c>
     </row>
     <row r="230" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A230" t="s">
+      <c r="A230" s="8" t="s">
         <v>246</v>
       </c>
       <c r="B230" t="s">
@@ -9213,7 +9367,7 @@
       </c>
     </row>
     <row r="231" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A231" t="s">
+      <c r="A231" s="8" t="s">
         <v>247</v>
       </c>
       <c r="B231" t="s">
@@ -9239,7 +9393,7 @@
       </c>
     </row>
     <row r="232" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A232" t="s">
+      <c r="A232" s="8" t="s">
         <v>248</v>
       </c>
       <c r="B232" t="s">
@@ -9265,7 +9419,7 @@
       </c>
     </row>
     <row r="233" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A233" t="s">
+      <c r="A233" s="8" t="s">
         <v>249</v>
       </c>
       <c r="B233" t="s">
@@ -9291,7 +9445,7 @@
       </c>
     </row>
     <row r="234" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A234" t="s">
+      <c r="A234" s="8" t="s">
         <v>250</v>
       </c>
       <c r="B234" t="s">
@@ -9317,7 +9471,7 @@
       </c>
     </row>
     <row r="235" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A235" t="s">
+      <c r="A235" s="8" t="s">
         <v>251</v>
       </c>
       <c r="B235" t="s">
@@ -9343,7 +9497,7 @@
       </c>
     </row>
     <row r="236" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A236" t="s">
+      <c r="A236" s="8" t="s">
         <v>252</v>
       </c>
       <c r="B236" t="s">
@@ -9369,7 +9523,7 @@
       </c>
     </row>
     <row r="237" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A237" t="s">
+      <c r="A237" s="8" t="s">
         <v>253</v>
       </c>
       <c r="B237" t="s">
@@ -9395,7 +9549,7 @@
       </c>
     </row>
     <row r="238" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A238" t="s">
+      <c r="A238" s="8" t="s">
         <v>254</v>
       </c>
       <c r="B238" t="s">
@@ -9421,7 +9575,7 @@
       </c>
     </row>
     <row r="239" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A239" t="s">
+      <c r="A239" s="8" t="s">
         <v>255</v>
       </c>
       <c r="B239" t="s">
@@ -9447,7 +9601,7 @@
       </c>
     </row>
     <row r="240" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A240" t="s">
+      <c r="A240" s="8" t="s">
         <v>256</v>
       </c>
       <c r="B240" t="s">
@@ -9473,7 +9627,7 @@
       </c>
     </row>
     <row r="241" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A241" t="s">
+      <c r="A241" s="8" t="s">
         <v>257</v>
       </c>
       <c r="B241" t="s">
@@ -9499,7 +9653,7 @@
       </c>
     </row>
     <row r="242" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A242" t="s">
+      <c r="A242" s="8" t="s">
         <v>258</v>
       </c>
       <c r="B242" t="s">
@@ -9525,7 +9679,7 @@
       </c>
     </row>
     <row r="243" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A243" t="s">
+      <c r="A243" s="8" t="s">
         <v>259</v>
       </c>
       <c r="B243" t="s">
@@ -9551,7 +9705,7 @@
       </c>
     </row>
     <row r="244" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A244" t="s">
+      <c r="A244" s="8" t="s">
         <v>260</v>
       </c>
       <c r="B244" t="s">
@@ -9577,7 +9731,7 @@
       </c>
     </row>
     <row r="245" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A245" t="s">
+      <c r="A245" s="8" t="s">
         <v>261</v>
       </c>
       <c r="B245" t="s">
@@ -9603,7 +9757,7 @@
       </c>
     </row>
     <row r="246" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A246" t="s">
+      <c r="A246" s="8" t="s">
         <v>262</v>
       </c>
       <c r="B246" t="s">
@@ -9629,7 +9783,7 @@
       </c>
     </row>
     <row r="247" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A247" t="s">
+      <c r="A247" s="8" t="s">
         <v>263</v>
       </c>
       <c r="B247" t="s">
@@ -9655,7 +9809,7 @@
       </c>
     </row>
     <row r="248" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A248" t="s">
+      <c r="A248" s="8" t="s">
         <v>264</v>
       </c>
       <c r="B248" t="s">
@@ -9681,7 +9835,7 @@
       </c>
     </row>
     <row r="249" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A249" t="s">
+      <c r="A249" s="8" t="s">
         <v>265</v>
       </c>
       <c r="B249" t="s">
@@ -9707,7 +9861,7 @@
       </c>
     </row>
     <row r="250" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A250" t="s">
+      <c r="A250" s="8" t="s">
         <v>266</v>
       </c>
       <c r="B250" t="s">
@@ -9733,7 +9887,7 @@
       </c>
     </row>
     <row r="251" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A251" t="s">
+      <c r="A251" s="8" t="s">
         <v>267</v>
       </c>
       <c r="B251" t="s">
@@ -9759,7 +9913,7 @@
       </c>
     </row>
     <row r="252" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A252" t="s">
+      <c r="A252" s="8" t="s">
         <v>268</v>
       </c>
       <c r="B252" t="s">
@@ -9785,7 +9939,7 @@
       </c>
     </row>
     <row r="253" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A253" t="s">
+      <c r="A253" s="8" t="s">
         <v>269</v>
       </c>
       <c r="B253" t="s">
@@ -9811,7 +9965,7 @@
       </c>
     </row>
     <row r="254" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A254" t="s">
+      <c r="A254" s="8" t="s">
         <v>270</v>
       </c>
       <c r="B254" t="s">
@@ -9837,7 +9991,7 @@
       </c>
     </row>
     <row r="255" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A255" t="s">
+      <c r="A255" s="8" t="s">
         <v>271</v>
       </c>
       <c r="B255" t="s">
@@ -9863,7 +10017,7 @@
       </c>
     </row>
     <row r="256" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A256" t="s">
+      <c r="A256" s="8" t="s">
         <v>272</v>
       </c>
       <c r="B256" t="s">
@@ -9889,7 +10043,7 @@
       </c>
     </row>
     <row r="257" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A257" t="s">
+      <c r="A257" s="8" t="s">
         <v>273</v>
       </c>
       <c r="B257" t="s">
@@ -9915,7 +10069,7 @@
       </c>
     </row>
     <row r="258" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A258" t="s">
+      <c r="A258" s="8" t="s">
         <v>274</v>
       </c>
       <c r="B258" t="s">
@@ -9941,7 +10095,7 @@
       </c>
     </row>
     <row r="259" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A259" t="s">
+      <c r="A259" s="8" t="s">
         <v>275</v>
       </c>
       <c r="B259" t="s">
@@ -9967,7 +10121,7 @@
       </c>
     </row>
     <row r="260" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A260" t="s">
+      <c r="A260" s="8" t="s">
         <v>276</v>
       </c>
       <c r="B260" t="s">
@@ -9993,7 +10147,7 @@
       </c>
     </row>
     <row r="261" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A261" t="s">
+      <c r="A261" s="8" t="s">
         <v>277</v>
       </c>
       <c r="B261" t="s">
@@ -10019,7 +10173,7 @@
       </c>
     </row>
     <row r="262" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A262" t="s">
+      <c r="A262" s="8" t="s">
         <v>278</v>
       </c>
       <c r="B262" t="s">
@@ -10045,7 +10199,7 @@
       </c>
     </row>
     <row r="263" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A263" t="s">
+      <c r="A263" s="8" t="s">
         <v>279</v>
       </c>
       <c r="B263" t="s">
@@ -10071,7 +10225,7 @@
       </c>
     </row>
     <row r="264" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A264" t="s">
+      <c r="A264" s="8" t="s">
         <v>280</v>
       </c>
       <c r="B264" t="s">
@@ -10097,7 +10251,7 @@
       </c>
     </row>
     <row r="265" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A265" t="s">
+      <c r="A265" s="8" t="s">
         <v>281</v>
       </c>
       <c r="B265" t="s">
@@ -10123,7 +10277,7 @@
       </c>
     </row>
     <row r="266" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A266" t="s">
+      <c r="A266" s="8" t="s">
         <v>282</v>
       </c>
       <c r="B266" t="s">
@@ -10149,7 +10303,7 @@
       </c>
     </row>
     <row r="267" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A267" t="s">
+      <c r="A267" s="8" t="s">
         <v>283</v>
       </c>
       <c r="B267" t="s">
@@ -10175,7 +10329,7 @@
       </c>
     </row>
     <row r="268" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A268" t="s">
+      <c r="A268" s="8" t="s">
         <v>284</v>
       </c>
       <c r="B268" t="s">
@@ -10201,7 +10355,7 @@
       </c>
     </row>
     <row r="269" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A269" t="s">
+      <c r="A269" s="8" t="s">
         <v>285</v>
       </c>
       <c r="B269" t="s">
@@ -10227,7 +10381,7 @@
       </c>
     </row>
     <row r="270" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A270" t="s">
+      <c r="A270" s="8" t="s">
         <v>286</v>
       </c>
       <c r="B270" t="s">
@@ -10253,7 +10407,7 @@
       </c>
     </row>
     <row r="271" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A271" t="s">
+      <c r="A271" s="8" t="s">
         <v>287</v>
       </c>
       <c r="B271" t="s">
@@ -10279,7 +10433,7 @@
       </c>
     </row>
     <row r="272" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A272" t="s">
+      <c r="A272" s="8" t="s">
         <v>287</v>
       </c>
       <c r="B272" t="s">
@@ -10305,7 +10459,7 @@
       </c>
     </row>
     <row r="273" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A273" t="s">
+      <c r="A273" s="8" t="s">
         <v>287</v>
       </c>
       <c r="B273" t="s">
@@ -10331,7 +10485,7 @@
       </c>
     </row>
     <row r="274" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A274" t="s">
+      <c r="A274" s="8" t="s">
         <v>288</v>
       </c>
       <c r="B274" t="s">
@@ -10357,7 +10511,7 @@
       </c>
     </row>
     <row r="275" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A275" t="s">
+      <c r="A275" s="8" t="s">
         <v>289</v>
       </c>
       <c r="B275" t="s">
@@ -10383,7 +10537,7 @@
       </c>
     </row>
     <row r="276" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A276" t="s">
+      <c r="A276" s="8" t="s">
         <v>290</v>
       </c>
       <c r="B276" t="s">
@@ -10409,7 +10563,7 @@
       </c>
     </row>
     <row r="277" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A277" t="s">
+      <c r="A277" s="8" t="s">
         <v>291</v>
       </c>
       <c r="B277" t="s">
@@ -10435,7 +10589,7 @@
       </c>
     </row>
     <row r="278" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A278" t="s">
+      <c r="A278" s="8" t="s">
         <v>292</v>
       </c>
       <c r="B278" t="s">
@@ -10461,7 +10615,7 @@
       </c>
     </row>
     <row r="279" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A279" t="s">
+      <c r="A279" s="8" t="s">
         <v>293</v>
       </c>
       <c r="B279" t="s">
@@ -10487,7 +10641,7 @@
       </c>
     </row>
     <row r="280" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A280" t="s">
+      <c r="A280" s="8" t="s">
         <v>294</v>
       </c>
       <c r="B280" t="s">
@@ -10513,7 +10667,7 @@
       </c>
     </row>
     <row r="281" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A281" t="s">
+      <c r="A281" s="8" t="s">
         <v>295</v>
       </c>
       <c r="B281" t="s">
@@ -10539,7 +10693,7 @@
       </c>
     </row>
     <row r="282" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A282" t="s">
+      <c r="A282" s="8" t="s">
         <v>296</v>
       </c>
       <c r="B282" t="s">
@@ -10565,7 +10719,7 @@
       </c>
     </row>
     <row r="283" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A283" t="s">
+      <c r="A283" s="8" t="s">
         <v>297</v>
       </c>
       <c r="B283" t="s">
@@ -10591,7 +10745,7 @@
       </c>
     </row>
     <row r="284" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A284" t="s">
+      <c r="A284" s="8" t="s">
         <v>298</v>
       </c>
       <c r="B284" t="s">
@@ -10617,7 +10771,7 @@
       </c>
     </row>
     <row r="285" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A285" t="s">
+      <c r="A285" s="8" t="s">
         <v>299</v>
       </c>
       <c r="B285" t="s">
@@ -10643,7 +10797,7 @@
       </c>
     </row>
     <row r="286" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A286" t="s">
+      <c r="A286" s="8" t="s">
         <v>300</v>
       </c>
       <c r="B286" t="s">
@@ -10669,7 +10823,7 @@
       </c>
     </row>
     <row r="287" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A287" t="s">
+      <c r="A287" s="8" t="s">
         <v>301</v>
       </c>
       <c r="B287" t="s">
@@ -10695,7 +10849,7 @@
       </c>
     </row>
     <row r="288" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A288" t="s">
+      <c r="A288" s="8" t="s">
         <v>302</v>
       </c>
       <c r="B288" t="s">
@@ -10721,7 +10875,7 @@
       </c>
     </row>
     <row r="289" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A289" t="s">
+      <c r="A289" s="8" t="s">
         <v>303</v>
       </c>
       <c r="B289" t="s">
@@ -10747,7 +10901,7 @@
       </c>
     </row>
     <row r="290" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A290" t="s">
+      <c r="A290" s="8" t="s">
         <v>304</v>
       </c>
       <c r="B290" t="s">
@@ -10773,7 +10927,7 @@
       </c>
     </row>
     <row r="291" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A291" t="s">
+      <c r="A291" s="8" t="s">
         <v>305</v>
       </c>
       <c r="B291" t="s">
@@ -10799,7 +10953,7 @@
       </c>
     </row>
     <row r="292" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A292" t="s">
+      <c r="A292" s="8" t="s">
         <v>306</v>
       </c>
       <c r="B292" t="s">
@@ -10825,7 +10979,7 @@
       </c>
     </row>
     <row r="293" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A293" t="s">
+      <c r="A293" s="8" t="s">
         <v>307</v>
       </c>
       <c r="B293" t="s">
@@ -10851,7 +11005,7 @@
       </c>
     </row>
     <row r="294" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A294" t="s">
+      <c r="A294" s="8" t="s">
         <v>308</v>
       </c>
       <c r="B294" t="s">
@@ -10877,7 +11031,7 @@
       </c>
     </row>
     <row r="295" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A295" t="s">
+      <c r="A295" s="8" t="s">
         <v>309</v>
       </c>
       <c r="B295" t="s">
@@ -10903,7 +11057,7 @@
       </c>
     </row>
     <row r="296" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A296" t="s">
+      <c r="A296" s="8" t="s">
         <v>310</v>
       </c>
       <c r="B296" t="s">
@@ -10929,7 +11083,7 @@
       </c>
     </row>
     <row r="297" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A297" t="s">
+      <c r="A297" s="8" t="s">
         <v>311</v>
       </c>
       <c r="B297" t="s">
@@ -10955,7 +11109,7 @@
       </c>
     </row>
     <row r="298" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A298" t="s">
+      <c r="A298" s="8" t="s">
         <v>312</v>
       </c>
       <c r="B298" t="s">
@@ -10981,7 +11135,7 @@
       </c>
     </row>
     <row r="299" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A299" t="s">
+      <c r="A299" s="8" t="s">
         <v>313</v>
       </c>
       <c r="B299" t="s">
@@ -11007,7 +11161,7 @@
       </c>
     </row>
     <row r="300" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A300" t="s">
+      <c r="A300" s="8" t="s">
         <v>314</v>
       </c>
       <c r="B300" t="s">
@@ -11033,7 +11187,7 @@
       </c>
     </row>
     <row r="301" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A301" t="s">
+      <c r="A301" s="8" t="s">
         <v>315</v>
       </c>
       <c r="B301" t="s">
@@ -11059,7 +11213,7 @@
       </c>
     </row>
     <row r="302" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A302" t="s">
+      <c r="A302" s="8" t="s">
         <v>316</v>
       </c>
       <c r="B302" t="s">
@@ -11085,7 +11239,7 @@
       </c>
     </row>
     <row r="303" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A303" t="s">
+      <c r="A303" s="8" t="s">
         <v>317</v>
       </c>
       <c r="B303" t="s">
@@ -11111,7 +11265,7 @@
       </c>
     </row>
     <row r="304" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A304" t="s">
+      <c r="A304" s="8" t="s">
         <v>317</v>
       </c>
       <c r="B304" t="s">
@@ -11137,7 +11291,7 @@
       </c>
     </row>
     <row r="305" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A305" t="s">
+      <c r="A305" s="8" t="s">
         <v>318</v>
       </c>
       <c r="B305" t="s">
@@ -11163,7 +11317,7 @@
       </c>
     </row>
     <row r="306" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A306" t="s">
+      <c r="A306" s="8" t="s">
         <v>319</v>
       </c>
       <c r="B306" t="s">
@@ -11189,7 +11343,7 @@
       </c>
     </row>
     <row r="307" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A307" t="s">
+      <c r="A307" s="8" t="s">
         <v>320</v>
       </c>
       <c r="B307" t="s">
@@ -11215,7 +11369,7 @@
       </c>
     </row>
     <row r="308" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A308" t="s">
+      <c r="A308" s="8" t="s">
         <v>321</v>
       </c>
       <c r="B308" t="s">
@@ -11241,7 +11395,7 @@
       </c>
     </row>
     <row r="309" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A309" t="s">
+      <c r="A309" s="8" t="s">
         <v>322</v>
       </c>
       <c r="B309" t="s">
@@ -11267,7 +11421,7 @@
       </c>
     </row>
     <row r="310" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A310" t="s">
+      <c r="A310" s="8" t="s">
         <v>323</v>
       </c>
       <c r="B310" t="s">
@@ -11293,7 +11447,7 @@
       </c>
     </row>
     <row r="311" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A311" t="s">
+      <c r="A311" s="8" t="s">
         <v>324</v>
       </c>
       <c r="B311" t="s">
@@ -11319,7 +11473,7 @@
       </c>
     </row>
     <row r="312" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A312" t="s">
+      <c r="A312" s="8" t="s">
         <v>325</v>
       </c>
       <c r="B312" t="s">
@@ -11345,7 +11499,7 @@
       </c>
     </row>
     <row r="313" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A313" t="s">
+      <c r="A313" s="8" t="s">
         <v>326</v>
       </c>
       <c r="B313" t="s">
@@ -11371,7 +11525,7 @@
       </c>
     </row>
     <row r="314" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A314" t="s">
+      <c r="A314" s="8" t="s">
         <v>327</v>
       </c>
       <c r="B314" t="s">
@@ -11397,7 +11551,7 @@
       </c>
     </row>
     <row r="315" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A315" t="s">
+      <c r="A315" s="8" t="s">
         <v>328</v>
       </c>
       <c r="B315" t="s">
@@ -11423,7 +11577,7 @@
       </c>
     </row>
     <row r="316" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A316" t="s">
+      <c r="A316" s="8" t="s">
         <v>329</v>
       </c>
       <c r="B316" t="s">
@@ -11449,7 +11603,7 @@
       </c>
     </row>
     <row r="317" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A317" t="s">
+      <c r="A317" s="8" t="s">
         <v>330</v>
       </c>
       <c r="B317" t="s">
@@ -11475,7 +11629,7 @@
       </c>
     </row>
     <row r="318" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A318" t="s">
+      <c r="A318" s="8" t="s">
         <v>331</v>
       </c>
       <c r="B318" t="s">
@@ -11501,7 +11655,7 @@
       </c>
     </row>
     <row r="319" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A319" t="s">
+      <c r="A319" s="8" t="s">
         <v>332</v>
       </c>
       <c r="B319" t="s">
@@ -11527,7 +11681,7 @@
       </c>
     </row>
     <row r="320" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A320" t="s">
+      <c r="A320" s="8" t="s">
         <v>333</v>
       </c>
       <c r="B320" t="s">
@@ -11553,7 +11707,7 @@
       </c>
     </row>
     <row r="321" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A321" t="s">
+      <c r="A321" s="8" t="s">
         <v>334</v>
       </c>
       <c r="B321" t="s">
@@ -11579,7 +11733,7 @@
       </c>
     </row>
     <row r="322" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A322" t="s">
+      <c r="A322" s="8" t="s">
         <v>335</v>
       </c>
       <c r="B322" t="s">
@@ -11605,7 +11759,7 @@
       </c>
     </row>
     <row r="323" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A323" t="s">
+      <c r="A323" s="8" t="s">
         <v>336</v>
       </c>
       <c r="B323" t="s">
@@ -11631,7 +11785,7 @@
       </c>
     </row>
     <row r="324" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A324" t="s">
+      <c r="A324" s="8" t="s">
         <v>337</v>
       </c>
       <c r="B324" t="s">
@@ -11657,7 +11811,7 @@
       </c>
     </row>
     <row r="325" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A325" t="s">
+      <c r="A325" s="8" t="s">
         <v>338</v>
       </c>
       <c r="B325" t="s">
@@ -11683,7 +11837,7 @@
       </c>
     </row>
     <row r="326" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A326" t="s">
+      <c r="A326" s="8" t="s">
         <v>339</v>
       </c>
       <c r="B326" t="s">
@@ -11709,7 +11863,7 @@
       </c>
     </row>
     <row r="327" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A327" t="s">
+      <c r="A327" s="8" t="s">
         <v>340</v>
       </c>
       <c r="B327" t="s">
@@ -11735,7 +11889,7 @@
       </c>
     </row>
     <row r="328" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A328" t="s">
+      <c r="A328" s="8" t="s">
         <v>341</v>
       </c>
       <c r="B328" t="s">
@@ -11761,7 +11915,7 @@
       </c>
     </row>
     <row r="329" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A329" t="s">
+      <c r="A329" s="8" t="s">
         <v>342</v>
       </c>
       <c r="B329" t="s">
@@ -11787,7 +11941,7 @@
       </c>
     </row>
     <row r="330" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A330" t="s">
+      <c r="A330" s="8" t="s">
         <v>343</v>
       </c>
       <c r="B330" t="s">
@@ -11813,7 +11967,7 @@
       </c>
     </row>
     <row r="331" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A331" t="s">
+      <c r="A331" s="8" t="s">
         <v>344</v>
       </c>
       <c r="B331" t="s">
@@ -11839,7 +11993,7 @@
       </c>
     </row>
     <row r="332" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A332" t="s">
+      <c r="A332" s="8" t="s">
         <v>345</v>
       </c>
       <c r="B332" t="s">
@@ -11865,7 +12019,7 @@
       </c>
     </row>
     <row r="333" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A333" t="s">
+      <c r="A333" s="8" t="s">
         <v>346</v>
       </c>
       <c r="B333" t="s">
@@ -11891,7 +12045,7 @@
       </c>
     </row>
     <row r="334" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A334" t="s">
+      <c r="A334" s="8" t="s">
         <v>347</v>
       </c>
       <c r="B334" t="s">
@@ -11917,7 +12071,7 @@
       </c>
     </row>
     <row r="335" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A335" t="s">
+      <c r="A335" s="8" t="s">
         <v>348</v>
       </c>
       <c r="B335" t="s">
@@ -11943,7 +12097,7 @@
       </c>
     </row>
     <row r="336" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A336" t="s">
+      <c r="A336" s="8" t="s">
         <v>349</v>
       </c>
       <c r="B336" t="s">
@@ -11969,7 +12123,7 @@
       </c>
     </row>
     <row r="337" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A337" t="s">
+      <c r="A337" s="8" t="s">
         <v>350</v>
       </c>
       <c r="B337" t="s">
@@ -11995,7 +12149,7 @@
       </c>
     </row>
     <row r="338" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A338" t="s">
+      <c r="A338" s="8" t="s">
         <v>351</v>
       </c>
       <c r="B338" t="s">
@@ -12021,7 +12175,7 @@
       </c>
     </row>
     <row r="339" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A339" t="s">
+      <c r="A339" s="8" t="s">
         <v>352</v>
       </c>
       <c r="B339" t="s">
@@ -12047,7 +12201,7 @@
       </c>
     </row>
     <row r="340" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A340" t="s">
+      <c r="A340" s="8" t="s">
         <v>353</v>
       </c>
       <c r="B340" t="s">
@@ -12073,7 +12227,7 @@
       </c>
     </row>
     <row r="341" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A341" t="s">
+      <c r="A341" s="8" t="s">
         <v>354</v>
       </c>
       <c r="B341" t="s">
@@ -12099,7 +12253,7 @@
       </c>
     </row>
     <row r="342" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A342" t="s">
+      <c r="A342" s="8" t="s">
         <v>355</v>
       </c>
       <c r="B342" t="s">
@@ -12125,7 +12279,7 @@
       </c>
     </row>
     <row r="343" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A343" t="s">
+      <c r="A343" s="8" t="s">
         <v>356</v>
       </c>
       <c r="B343" t="s">
@@ -12151,7 +12305,7 @@
       </c>
     </row>
     <row r="344" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A344" t="s">
+      <c r="A344" s="8" t="s">
         <v>357</v>
       </c>
       <c r="B344" t="s">
@@ -12177,7 +12331,7 @@
       </c>
     </row>
     <row r="345" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A345" t="s">
+      <c r="A345" s="8" t="s">
         <v>358</v>
       </c>
       <c r="B345" t="s">
@@ -12203,7 +12357,7 @@
       </c>
     </row>
     <row r="346" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A346" t="s">
+      <c r="A346" s="8" t="s">
         <v>359</v>
       </c>
       <c r="B346" t="s">
@@ -12229,7 +12383,7 @@
       </c>
     </row>
     <row r="347" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A347" t="s">
+      <c r="A347" s="8" t="s">
         <v>360</v>
       </c>
       <c r="B347" t="s">
@@ -12255,7 +12409,7 @@
       </c>
     </row>
     <row r="348" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A348" t="s">
+      <c r="A348" s="8" t="s">
         <v>361</v>
       </c>
       <c r="B348" t="s">
@@ -12281,7 +12435,7 @@
       </c>
     </row>
     <row r="349" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A349" t="s">
+      <c r="A349" s="8" t="s">
         <v>362</v>
       </c>
       <c r="B349" t="s">
@@ -12307,7 +12461,7 @@
       </c>
     </row>
     <row r="350" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A350" t="s">
+      <c r="A350" s="8" t="s">
         <v>363</v>
       </c>
       <c r="B350" t="s">
@@ -12333,7 +12487,7 @@
       </c>
     </row>
     <row r="351" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A351" t="s">
+      <c r="A351" s="8" t="s">
         <v>364</v>
       </c>
       <c r="B351" t="s">
@@ -12359,7 +12513,7 @@
       </c>
     </row>
     <row r="352" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A352" t="s">
+      <c r="A352" s="8" t="s">
         <v>365</v>
       </c>
       <c r="B352" t="s">
@@ -12385,7 +12539,7 @@
       </c>
     </row>
     <row r="353" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A353" t="s">
+      <c r="A353" s="8" t="s">
         <v>366</v>
       </c>
       <c r="B353" t="s">
@@ -12411,7 +12565,7 @@
       </c>
     </row>
     <row r="354" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A354" t="s">
+      <c r="A354" s="8" t="s">
         <v>367</v>
       </c>
       <c r="B354" t="s">
@@ -12437,7 +12591,7 @@
       </c>
     </row>
     <row r="355" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A355" t="s">
+      <c r="A355" s="8" t="s">
         <v>368</v>
       </c>
       <c r="B355" t="s">
@@ -12463,7 +12617,7 @@
       </c>
     </row>
     <row r="356" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A356" t="s">
+      <c r="A356" s="8" t="s">
         <v>369</v>
       </c>
       <c r="B356" t="s">
@@ -12489,7 +12643,7 @@
       </c>
     </row>
     <row r="357" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A357" t="s">
+      <c r="A357" s="8" t="s">
         <v>370</v>
       </c>
       <c r="B357" t="s">
@@ -12515,7 +12669,7 @@
       </c>
     </row>
     <row r="358" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A358" t="s">
+      <c r="A358" s="8" t="s">
         <v>371</v>
       </c>
       <c r="B358" t="s">
@@ -12541,7 +12695,7 @@
       </c>
     </row>
     <row r="359" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A359" t="s">
+      <c r="A359" s="8" t="s">
         <v>372</v>
       </c>
       <c r="B359" t="s">
@@ -12567,7 +12721,7 @@
       </c>
     </row>
     <row r="360" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A360" t="s">
+      <c r="A360" s="8" t="s">
         <v>373</v>
       </c>
       <c r="B360" t="s">
@@ -12593,7 +12747,7 @@
       </c>
     </row>
     <row r="361" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A361" t="s">
+      <c r="A361" s="8" t="s">
         <v>374</v>
       </c>
       <c r="B361" t="s">
@@ -12619,7 +12773,7 @@
       </c>
     </row>
     <row r="362" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A362" t="s">
+      <c r="A362" s="8" t="s">
         <v>375</v>
       </c>
       <c r="B362" t="s">
@@ -12645,7 +12799,7 @@
       </c>
     </row>
     <row r="363" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A363" t="s">
+      <c r="A363" s="8" t="s">
         <v>376</v>
       </c>
       <c r="B363" t="s">
@@ -12671,7 +12825,7 @@
       </c>
     </row>
     <row r="364" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A364" t="s">
+      <c r="A364" s="8" t="s">
         <v>377</v>
       </c>
       <c r="B364" t="s">
@@ -12697,7 +12851,7 @@
       </c>
     </row>
     <row r="365" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A365" t="s">
+      <c r="A365" s="8" t="s">
         <v>378</v>
       </c>
       <c r="B365" t="s">
@@ -12723,7 +12877,7 @@
       </c>
     </row>
     <row r="366" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A366" t="s">
+      <c r="A366" s="8" t="s">
         <v>379</v>
       </c>
       <c r="B366" t="s">
@@ -12749,7 +12903,7 @@
       </c>
     </row>
     <row r="367" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A367" t="s">
+      <c r="A367" s="8" t="s">
         <v>380</v>
       </c>
       <c r="B367" t="s">
@@ -12775,7 +12929,7 @@
       </c>
     </row>
     <row r="368" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A368" t="s">
+      <c r="A368" s="8" t="s">
         <v>381</v>
       </c>
       <c r="B368" t="s">
@@ -12801,7 +12955,7 @@
       </c>
     </row>
     <row r="369" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A369" t="s">
+      <c r="A369" s="8" t="s">
         <v>382</v>
       </c>
       <c r="B369" t="s">
@@ -12827,7 +12981,7 @@
       </c>
     </row>
     <row r="370" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A370" t="s">
+      <c r="A370" s="8" t="s">
         <v>383</v>
       </c>
       <c r="B370" t="s">
@@ -12853,7 +13007,7 @@
       </c>
     </row>
     <row r="371" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A371" t="s">
+      <c r="A371" s="8" t="s">
         <v>384</v>
       </c>
       <c r="B371" t="s">
@@ -12879,7 +13033,7 @@
       </c>
     </row>
     <row r="372" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A372" t="s">
+      <c r="A372" s="8" t="s">
         <v>385</v>
       </c>
       <c r="B372" t="s">
@@ -12905,7 +13059,7 @@
       </c>
     </row>
     <row r="373" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A373" t="s">
+      <c r="A373" s="8" t="s">
         <v>386</v>
       </c>
       <c r="B373" t="s">
@@ -12931,7 +13085,7 @@
       </c>
     </row>
     <row r="374" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A374" t="s">
+      <c r="A374" s="8" t="s">
         <v>387</v>
       </c>
       <c r="B374" t="s">
@@ -12957,7 +13111,7 @@
       </c>
     </row>
     <row r="375" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A375" t="s">
+      <c r="A375" s="8" t="s">
         <v>388</v>
       </c>
       <c r="B375" t="s">
@@ -12983,7 +13137,7 @@
       </c>
     </row>
     <row r="376" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A376" t="s">
+      <c r="A376" s="8" t="s">
         <v>389</v>
       </c>
       <c r="B376" t="s">
@@ -13009,7 +13163,7 @@
       </c>
     </row>
     <row r="377" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A377" t="s">
+      <c r="A377" s="8" t="s">
         <v>390</v>
       </c>
       <c r="B377" t="s">
@@ -13035,7 +13189,7 @@
       </c>
     </row>
     <row r="378" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A378" t="s">
+      <c r="A378" s="8" t="s">
         <v>391</v>
       </c>
       <c r="B378" t="s">
@@ -13061,7 +13215,7 @@
       </c>
     </row>
     <row r="379" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A379" t="s">
+      <c r="A379" s="8" t="s">
         <v>392</v>
       </c>
       <c r="B379" t="s">
@@ -13087,7 +13241,7 @@
       </c>
     </row>
     <row r="380" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A380" t="s">
+      <c r="A380" s="8" t="s">
         <v>393</v>
       </c>
       <c r="B380" t="s">
@@ -13113,7 +13267,7 @@
       </c>
     </row>
     <row r="381" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A381" t="s">
+      <c r="A381" s="8" t="s">
         <v>394</v>
       </c>
       <c r="B381" t="s">
@@ -13139,7 +13293,7 @@
       </c>
     </row>
     <row r="382" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A382" t="s">
+      <c r="A382" s="8" t="s">
         <v>395</v>
       </c>
       <c r="B382" t="s">
@@ -13165,7 +13319,7 @@
       </c>
     </row>
     <row r="383" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A383" t="s">
+      <c r="A383" s="8" t="s">
         <v>396</v>
       </c>
       <c r="B383" t="s">
@@ -13191,7 +13345,7 @@
       </c>
     </row>
     <row r="384" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A384" t="s">
+      <c r="A384" s="8" t="s">
         <v>397</v>
       </c>
       <c r="B384" t="s">
@@ -13217,7 +13371,7 @@
       </c>
     </row>
     <row r="385" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A385" t="s">
+      <c r="A385" s="8" t="s">
         <v>398</v>
       </c>
       <c r="B385" t="s">
@@ -13243,7 +13397,7 @@
       </c>
     </row>
     <row r="386" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A386" t="s">
+      <c r="A386" s="8" t="s">
         <v>399</v>
       </c>
       <c r="B386" t="s">
@@ -13269,7 +13423,7 @@
       </c>
     </row>
     <row r="387" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A387" t="s">
+      <c r="A387" s="8" t="s">
         <v>400</v>
       </c>
       <c r="B387" t="s">
@@ -13295,7 +13449,7 @@
       </c>
     </row>
     <row r="388" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A388" t="s">
+      <c r="A388" s="8" t="s">
         <v>401</v>
       </c>
       <c r="B388" t="s">
@@ -13321,7 +13475,7 @@
       </c>
     </row>
     <row r="389" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A389" t="s">
+      <c r="A389" s="8" t="s">
         <v>402</v>
       </c>
       <c r="B389" t="s">
@@ -13347,7 +13501,7 @@
       </c>
     </row>
     <row r="390" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A390" t="s">
+      <c r="A390" s="8" t="s">
         <v>403</v>
       </c>
       <c r="B390" t="s">
@@ -13373,7 +13527,7 @@
       </c>
     </row>
     <row r="391" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A391" t="s">
+      <c r="A391" s="8" t="s">
         <v>404</v>
       </c>
       <c r="B391" t="s">
@@ -13399,7 +13553,7 @@
       </c>
     </row>
     <row r="392" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A392" t="s">
+      <c r="A392" s="8" t="s">
         <v>405</v>
       </c>
       <c r="B392" t="s">
@@ -13425,7 +13579,7 @@
       </c>
     </row>
     <row r="393" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A393" t="s">
+      <c r="A393" s="8" t="s">
         <v>406</v>
       </c>
       <c r="B393" t="s">
@@ -13451,7 +13605,7 @@
       </c>
     </row>
     <row r="394" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A394" t="s">
+      <c r="A394" s="8" t="s">
         <v>407</v>
       </c>
       <c r="B394" t="s">
@@ -13477,7 +13631,7 @@
       </c>
     </row>
     <row r="395" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A395" t="s">
+      <c r="A395" s="8" t="s">
         <v>408</v>
       </c>
       <c r="B395" t="s">
@@ -13503,7 +13657,7 @@
       </c>
     </row>
     <row r="396" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A396" t="s">
+      <c r="A396" s="8" t="s">
         <v>409</v>
       </c>
       <c r="B396" t="s">
@@ -13529,7 +13683,7 @@
       </c>
     </row>
     <row r="397" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A397" t="s">
+      <c r="A397" s="8" t="s">
         <v>410</v>
       </c>
       <c r="B397" t="s">
@@ -13555,7 +13709,7 @@
       </c>
     </row>
     <row r="398" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A398" t="s">
+      <c r="A398" s="8" t="s">
         <v>411</v>
       </c>
       <c r="B398" t="s">
@@ -13581,7 +13735,7 @@
       </c>
     </row>
     <row r="399" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A399" t="s">
+      <c r="A399" s="8" t="s">
         <v>412</v>
       </c>
       <c r="B399" t="s">
@@ -13607,7 +13761,7 @@
       </c>
     </row>
     <row r="400" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A400" t="s">
+      <c r="A400" s="8" t="s">
         <v>413</v>
       </c>
       <c r="B400" t="s">
@@ -13633,7 +13787,7 @@
       </c>
     </row>
     <row r="401" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A401" t="s">
+      <c r="A401" s="8" t="s">
         <v>414</v>
       </c>
       <c r="B401" t="s">
@@ -13659,7 +13813,7 @@
       </c>
     </row>
     <row r="402" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A402" t="s">
+      <c r="A402" s="8" t="s">
         <v>415</v>
       </c>
       <c r="B402" t="s">
@@ -13685,7 +13839,7 @@
       </c>
     </row>
     <row r="403" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A403" t="s">
+      <c r="A403" s="8" t="s">
         <v>416</v>
       </c>
       <c r="B403" t="s">
@@ -13711,7 +13865,7 @@
       </c>
     </row>
     <row r="404" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A404" t="s">
+      <c r="A404" s="8" t="s">
         <v>417</v>
       </c>
       <c r="B404" t="s">
@@ -13737,7 +13891,7 @@
       </c>
     </row>
     <row r="405" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A405" t="s">
+      <c r="A405" s="8" t="s">
         <v>418</v>
       </c>
       <c r="B405" t="s">
@@ -13763,7 +13917,7 @@
       </c>
     </row>
     <row r="406" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A406" t="s">
+      <c r="A406" s="8" t="s">
         <v>419</v>
       </c>
       <c r="B406" t="s">
@@ -13789,7 +13943,7 @@
       </c>
     </row>
     <row r="407" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A407" t="s">
+      <c r="A407" s="8" t="s">
         <v>420</v>
       </c>
       <c r="B407" t="s">
@@ -13815,7 +13969,7 @@
       </c>
     </row>
     <row r="408" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A408" t="s">
+      <c r="A408" s="8" t="s">
         <v>421</v>
       </c>
       <c r="B408" t="s">
@@ -13841,7 +13995,7 @@
       </c>
     </row>
     <row r="409" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A409" t="s">
+      <c r="A409" s="8" t="s">
         <v>422</v>
       </c>
       <c r="B409" t="s">
@@ -13867,7 +14021,7 @@
       </c>
     </row>
     <row r="410" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A410" t="s">
+      <c r="A410" s="8" t="s">
         <v>423</v>
       </c>
       <c r="B410" t="s">
@@ -13893,7 +14047,7 @@
       </c>
     </row>
     <row r="411" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A411" t="s">
+      <c r="A411" s="8" t="s">
         <v>424</v>
       </c>
       <c r="B411" t="s">
@@ -13919,7 +14073,7 @@
       </c>
     </row>
     <row r="412" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A412" t="s">
+      <c r="A412" s="8" t="s">
         <v>425</v>
       </c>
       <c r="B412" t="s">
@@ -13945,7 +14099,7 @@
       </c>
     </row>
     <row r="413" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A413" t="s">
+      <c r="A413" s="8" t="s">
         <v>426</v>
       </c>
       <c r="B413" t="s">
@@ -13971,7 +14125,7 @@
       </c>
     </row>
     <row r="414" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A414" t="s">
+      <c r="A414" s="8" t="s">
         <v>427</v>
       </c>
       <c r="B414" t="s">
@@ -13997,7 +14151,7 @@
       </c>
     </row>
     <row r="415" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A415" t="s">
+      <c r="A415" s="8" t="s">
         <v>428</v>
       </c>
       <c r="B415" t="s">
@@ -14023,7 +14177,7 @@
       </c>
     </row>
     <row r="416" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A416" t="s">
+      <c r="A416" s="8" t="s">
         <v>429</v>
       </c>
       <c r="B416" t="s">
@@ -14049,7 +14203,7 @@
       </c>
     </row>
     <row r="417" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A417" t="s">
+      <c r="A417" s="8" t="s">
         <v>430</v>
       </c>
       <c r="B417" t="s">
@@ -14075,7 +14229,7 @@
       </c>
     </row>
     <row r="418" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A418" t="s">
+      <c r="A418" s="8" t="s">
         <v>431</v>
       </c>
       <c r="B418" t="s">
@@ -14101,7 +14255,7 @@
       </c>
     </row>
     <row r="419" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A419" t="s">
+      <c r="A419" s="8" t="s">
         <v>432</v>
       </c>
       <c r="B419" t="s">
@@ -14127,7 +14281,7 @@
       </c>
     </row>
     <row r="420" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A420" t="s">
+      <c r="A420" s="8" t="s">
         <v>433</v>
       </c>
       <c r="B420" t="s">
@@ -14153,7 +14307,7 @@
       </c>
     </row>
     <row r="421" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A421" t="s">
+      <c r="A421" s="8" t="s">
         <v>434</v>
       </c>
       <c r="B421" t="s">
@@ -14179,7 +14333,7 @@
       </c>
     </row>
     <row r="422" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A422" t="s">
+      <c r="A422" s="8" t="s">
         <v>435</v>
       </c>
       <c r="B422" t="s">
@@ -14205,7 +14359,7 @@
       </c>
     </row>
     <row r="423" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A423" t="s">
+      <c r="A423" s="8" t="s">
         <v>436</v>
       </c>
       <c r="B423" t="s">
@@ -14231,7 +14385,7 @@
       </c>
     </row>
     <row r="424" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A424" t="s">
+      <c r="A424" s="8" t="s">
         <v>437</v>
       </c>
       <c r="B424" t="s">
@@ -14257,7 +14411,7 @@
       </c>
     </row>
     <row r="425" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A425" t="s">
+      <c r="A425" s="8" t="s">
         <v>438</v>
       </c>
       <c r="B425" t="s">
@@ -14283,7 +14437,7 @@
       </c>
     </row>
     <row r="426" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A426" t="s">
+      <c r="A426" s="8" t="s">
         <v>439</v>
       </c>
       <c r="B426" t="s">
@@ -14309,7 +14463,7 @@
       </c>
     </row>
     <row r="427" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A427" t="s">
+      <c r="A427" s="8" t="s">
         <v>440</v>
       </c>
       <c r="B427" t="s">
@@ -14335,7 +14489,7 @@
       </c>
     </row>
     <row r="428" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A428" t="s">
+      <c r="A428" s="8" t="s">
         <v>441</v>
       </c>
       <c r="B428" t="s">
@@ -14361,7 +14515,7 @@
       </c>
     </row>
     <row r="429" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A429" t="s">
+      <c r="A429" s="8" t="s">
         <v>442</v>
       </c>
       <c r="B429" t="s">
@@ -14387,7 +14541,7 @@
       </c>
     </row>
     <row r="430" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A430" t="s">
+      <c r="A430" s="8" t="s">
         <v>443</v>
       </c>
       <c r="B430" t="s">
@@ -14413,7 +14567,7 @@
       </c>
     </row>
     <row r="431" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A431" t="s">
+      <c r="A431" s="8" t="s">
         <v>444</v>
       </c>
       <c r="B431" t="s">
@@ -14439,7 +14593,7 @@
       </c>
     </row>
     <row r="432" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A432" t="s">
+      <c r="A432" s="8" t="s">
         <v>445</v>
       </c>
       <c r="B432" t="s">
@@ -14465,7 +14619,7 @@
       </c>
     </row>
     <row r="433" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A433" t="s">
+      <c r="A433" s="8" t="s">
         <v>446</v>
       </c>
       <c r="B433" t="s">
@@ -14491,7 +14645,7 @@
       </c>
     </row>
     <row r="434" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A434" t="s">
+      <c r="A434" s="8" t="s">
         <v>447</v>
       </c>
       <c r="B434" t="s">
@@ -14517,7 +14671,7 @@
       </c>
     </row>
     <row r="435" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A435" t="s">
+      <c r="A435" s="8" t="s">
         <v>448</v>
       </c>
       <c r="B435" t="s">
@@ -14543,7 +14697,7 @@
       </c>
     </row>
     <row r="436" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A436" t="s">
+      <c r="A436" s="8" t="s">
         <v>449</v>
       </c>
       <c r="B436" t="s">
@@ -14569,7 +14723,7 @@
       </c>
     </row>
     <row r="437" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A437" t="s">
+      <c r="A437" s="8" t="s">
         <v>450</v>
       </c>
       <c r="B437" t="s">
@@ -14595,7 +14749,7 @@
       </c>
     </row>
     <row r="438" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A438" t="s">
+      <c r="A438" s="8" t="s">
         <v>451</v>
       </c>
       <c r="B438" t="s">
@@ -14621,7 +14775,7 @@
       </c>
     </row>
     <row r="439" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A439" t="s">
+      <c r="A439" s="8" t="s">
         <v>452</v>
       </c>
       <c r="B439" t="s">
@@ -14647,7 +14801,7 @@
       </c>
     </row>
     <row r="440" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A440" t="s">
+      <c r="A440" s="8" t="s">
         <v>453</v>
       </c>
       <c r="B440" t="s">
@@ -14673,7 +14827,7 @@
       </c>
     </row>
     <row r="441" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A441" t="s">
+      <c r="A441" s="8" t="s">
         <v>454</v>
       </c>
       <c r="B441" t="s">
@@ -14699,7 +14853,7 @@
       </c>
     </row>
     <row r="442" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A442" t="s">
+      <c r="A442" s="8" t="s">
         <v>455</v>
       </c>
       <c r="B442" t="s">
@@ -14725,7 +14879,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H442" xr:uid="{DC658449-BA0D-FB4C-A8FC-4A535294D741}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>